<commit_message>
feat: add LeetCode 209 (Minimum Size Subarray Sum) solution and update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\OneDrive\Desktop\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D9167D1-3A20-4D6E-80B9-046AB013538D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2362,7 +2362,9 @@
       <c r="E26" s="8"/>
     </row>
     <row r="27" spans="1:5" ht="14.4">
-      <c r="A27" s="6"/>
+      <c r="A27" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B27" s="9" t="s">
         <v>54</v>
       </c>

</xml_diff>

<commit_message>
feat: add Longest Substring with K Unique Characters solution and update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\OneDrive\Desktop\DSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{137844DF-967E-434A-B8F4-D3C7080ACA88}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2375,7 +2375,9 @@
       <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:5" ht="14.4">
-      <c r="A28" s="6"/>
+      <c r="A28" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B28" s="9" t="s">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
feat: add LeetCode 904 (Fruit Into Baskets) solution and update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{137844DF-967E-434A-B8F4-D3C7080ACA88}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEC4F5E5-9EF8-4FA6-A5C0-9E9CCA46AC9A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2388,7 +2388,9 @@
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="1:5" ht="14.4">
-      <c r="A29" s="6"/>
+      <c r="A29" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B29" s="9" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
feat: add LeetCode 3 (Longest Substring Without Repeating Characters) solution and update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEC4F5E5-9EF8-4FA6-A5C0-9E9CCA46AC9A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B09D4664-E3A0-4438-86F0-D0E35B3B3399}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2401,7 +2401,9 @@
       <c r="E29" s="8"/>
     </row>
     <row r="30" spans="1:5" ht="14.4">
-      <c r="A30" s="6"/>
+      <c r="A30" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B30" s="9" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 209 (Min Subarray Sum) & LC 76 (Min Window Substring) with updated README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B09D4664-E3A0-4438-86F0-D0E35B3B3399}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE9BC0EF-D643-4AAD-99F4-78AAFF54A189}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -1839,6 +1839,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -2414,7 +2418,9 @@
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="14.4">
-      <c r="A31" s="6"/>
+      <c r="A31" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B31" s="9" t="s">
         <v>62</v>
       </c>
@@ -2436,7 +2442,9 @@
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="14.4">
-      <c r="A33" s="6"/>
+      <c r="A33" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B33" s="9" t="s">
         <v>66</v>
       </c>
@@ -2447,7 +2455,9 @@
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="14.4">
-      <c r="A34" s="6"/>
+      <c r="A34" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B34" s="9" t="s">
         <v>67</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 876 Middle of Linked List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE9BC0EF-D643-4AAD-99F4-78AAFF54A189}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53800F27-0587-44A9-8839-1200EABA50FB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2256,7 +2256,9 @@
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A17" s="6"/>
+      <c r="A17" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B17" s="9" t="s">
         <v>35</v>
       </c>
@@ -2300,7 +2302,9 @@
       <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A21" s="6"/>
+      <c r="A21" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B21" s="9" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 142 Linked List Cycle II solution & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53800F27-0587-44A9-8839-1200EABA50FB}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E6A9A04-BF57-46CF-AC53-72BC56E027DA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2269,7 +2269,9 @@
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A18" s="6"/>
+      <c r="A18" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B18" s="9" t="s">
         <v>37</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 287 Find the Duplicate Number & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E6A9A04-BF57-46CF-AC53-72BC56E027DA}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7588416B-EA06-411D-9B0A-7DC1E6F5CE55}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2293,7 +2293,9 @@
       <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A20" s="6"/>
+      <c r="A20" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B20" s="9" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 202 Happy Number & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7588416B-EA06-411D-9B0A-7DC1E6F5CE55}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9ECAE436-42AE-4E9E-8A9C-75AD3EE715AA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2282,7 +2282,9 @@
       <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A19" s="6"/>
+      <c r="A19" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B19" s="9" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 1004 Max Consecutive Ones III & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9ECAE436-42AE-4E9E-8A9C-75AD3EE715AA}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F8962E8-B00F-42EA-B6FB-7718F4792134}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2441,7 +2441,9 @@
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="14.4">
-      <c r="A32" s="6"/>
+      <c r="A32" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B32" s="9" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
feat(arrays-hashing): add LC 53 Maximum Subarray (Kadane's Algorithm) & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F8962E8-B00F-42EA-B6FB-7718F4792134}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83696C83-A916-418D-90FF-075196AC6E80}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2188,7 +2188,9 @@
       <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
@@ -2522,7 +2524,9 @@
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="14.4">
-      <c r="A39" s="6"/>
+      <c r="A39" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B39" s="17" t="s">
         <v>76</v>
       </c>
@@ -2533,7 +2537,9 @@
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="14.4">
-      <c r="A40" s="6"/>
+      <c r="A40" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B40" s="9" t="s">
         <v>78</v>
       </c>
@@ -2544,7 +2550,9 @@
       <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" ht="14.4">
-      <c r="A41" s="6"/>
+      <c r="A41" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B41" s="17" t="s">
         <v>80</v>
       </c>

</xml_diff>

<commit_message>
feat(arrays-hashing): add LC 1749 Max Absolute Sum of Any Subarray & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83696C83-A916-418D-90FF-075196AC6E80}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D60ECECE-16B6-4785-9AD3-3A895B94323B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2574,7 +2574,9 @@
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="14.4">
-      <c r="A43" s="6"/>
+      <c r="A43" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B43" s="17" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
feat(arrays-hashing): add LC 1186 Max Subarray Sum with One Deletion & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D60ECECE-16B6-4785-9AD3-3A895B94323B}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3CAA36A-F727-46C5-89F9-6EA62C71C1A0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2563,7 +2563,9 @@
       <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5" ht="14.4">
-      <c r="A42" s="6"/>
+      <c r="A42" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B42" s="17" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
feat(arrays-hashing): add LC 918 Max Sum Circular Subarray & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3CAA36A-F727-46C5-89F9-6EA62C71C1A0}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5DC2DFA-1313-4095-967D-A80ED5979BF6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2589,7 +2589,9 @@
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="14.4">
-      <c r="A44" s="6"/>
+      <c r="A44" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B44" s="17" t="s">
         <v>86</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 457 Circular Array Loop & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5DC2DFA-1313-4095-967D-A80ED5979BF6}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF17E50B-25CC-47C0-B0E8-D7666DC2BC0F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2345,7 +2345,9 @@
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A24" s="6"/>
+      <c r="A24" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B24" s="6" t="s">
         <v>49</v>
       </c>

</xml_diff>

<commit_message>
feat(prefix-sum): add LC 560 Subarray Sum Equals K & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF17E50B-25CC-47C0-B0E8-D7666DC2BC0F}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD95A4D5-DA0E-498C-9BA8-E39DB34BB2DB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2613,7 +2613,9 @@
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="14.4">
-      <c r="A46" s="6"/>
+      <c r="A46" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B46" s="17" t="s">
         <v>89</v>
       </c>
@@ -2624,7 +2626,9 @@
       <c r="E46" s="8"/>
     </row>
     <row r="47" spans="1:5" ht="14.4">
-      <c r="A47" s="6"/>
+      <c r="A47" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B47" s="17" t="s">
         <v>91</v>
       </c>

</xml_diff>

<commit_message>
feat(prefix-sum): add LC 525 Contiguous Array & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD95A4D5-DA0E-498C-9BA8-E39DB34BB2DB}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B729F50-1AC2-4B1A-91B4-824B8EFEBFE7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2639,7 +2639,9 @@
       <c r="E47" s="8"/>
     </row>
     <row r="48" spans="1:5" ht="14.4">
-      <c r="A48" s="6"/>
+      <c r="A48" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B48" s="17" t="s">
         <v>93</v>
       </c>
@@ -2650,7 +2652,9 @@
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="14.4">
-      <c r="A49" s="6"/>
+      <c r="A49" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B49" s="17" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
feat(two-pointers): add LC 18 4Sum & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B729F50-1AC2-4B1A-91B4-824B8EFEBFE7}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B07557FD-2520-4E7A-95ED-52B3091CD598}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2214,7 +2214,9 @@
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A13" s="6"/>
+      <c r="A13" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B13" s="15" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
feat(two-pointers): add LC 844 Backspace String Compare & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B07557FD-2520-4E7A-95ED-52B3091CD598}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B71E093-ACF0-4847-8E82-7B515937ADE3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2227,7 +2227,9 @@
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A14" s="6"/>
+      <c r="A14" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B14" s="6" t="s">
         <v>29</v>
       </c>

</xml_diff>

<commit_message>
feat(two-pointers): add LC 581 Shortest Unsorted Subarray & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B71E093-ACF0-4847-8E82-7B515937ADE3}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16B74F9A-B86C-458C-9460-96833E9E28BB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2240,7 +2240,9 @@
       <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A15" s="6"/>
+      <c r="A15" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B15" s="6" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 234 Palindrome Linked List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16B74F9A-B86C-458C-9460-96833E9E28BB}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B9A0FEE-86FD-4857-821C-A8F8FDA3F6EE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2329,7 +2329,9 @@
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A22" s="6"/>
+      <c r="A22" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B22" s="6" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
feat(fast-slow-pointers): add LC 143 Reorder List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B9A0FEE-86FD-4857-821C-A8F8FDA3F6EE}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{886B899B-D3C0-4A5A-B98B-02AEC0330286}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2342,7 +2342,9 @@
       <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A23" s="6"/>
+      <c r="A23" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B23" s="6" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 567 Permutation in String & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{886B899B-D3C0-4A5A-B98B-02AEC0330286}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5387C190-EA44-47E8-9FA4-0AAF296ACF9D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2494,7 +2494,9 @@
       <c r="E34" s="8"/>
     </row>
     <row r="35" spans="1:5" ht="14.4">
-      <c r="A35" s="6"/>
+      <c r="A35" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B35" s="6" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 438 Find All Anagrams in a String & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5387C190-EA44-47E8-9FA4-0AAF296ACF9D}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A832CE56-6562-4F6D-BB12-7CDB7EEB28F4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2507,7 +2507,9 @@
       <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="14.4">
-      <c r="A36" s="6"/>
+      <c r="A36" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B36" s="6" t="s">
         <v>71</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 30 Substring with Concatenation of All Words & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A832CE56-6562-4F6D-BB12-7CDB7EEB28F4}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3050768F-A469-4A65-805F-196576AA54DA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2520,7 +2520,9 @@
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="14.4">
-      <c r="A37" s="6"/>
+      <c r="A37" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B37" s="6" t="s">
         <v>73</v>
       </c>

</xml_diff>

<commit_message>
feat(sliding-window): add LC 862 Shortest Subarray with Sum at Least K & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3050768F-A469-4A65-805F-196576AA54DA}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58126160-DEAA-4B94-A728-F620C071F321}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2681,7 +2681,9 @@
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="14.4">
-      <c r="A50" s="6"/>
+      <c r="A50" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B50" s="18" t="s">
         <v>97</v>
       </c>

</xml_diff>

<commit_message>
feat(prefix-sum): add LC 327 Count of Range Sum & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58126160-DEAA-4B94-A728-F620C071F321}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D04ED4B-16AD-4EBC-B19D-716E8372A033}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -1578,7 +1578,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1680,6 +1680,13 @@
       <color rgb="FF1155CC"/>
       <name val="Calibri, sans-serif"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -1773,10 +1780,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1822,8 +1830,10 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2687,14 +2697,16 @@
       <c r="B50" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="35" t="s">
         <v>98</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="14.4">
-      <c r="A51" s="6"/>
+      <c r="A51" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B51" s="18" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
feat(intervals): add LC 56 Merge Intervals & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D04ED4B-16AD-4EBC-B19D-716E8372A033}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E013D40-57BD-4773-A7FB-CB14D107FBB9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -1828,9 +1828,9 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2259,10 +2259,10 @@
       <c r="C15" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="33" t="s">
+      <c r="D15" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="34"/>
+      <c r="E15" s="35"/>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1">
       <c r="A16" s="6"/>
@@ -2697,7 +2697,7 @@
       <c r="B50" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="C50" s="35" t="s">
+      <c r="C50" s="33" t="s">
         <v>98</v>
       </c>
       <c r="D50" s="8"/>
@@ -2726,7 +2726,9 @@
       <c r="E52" s="8"/>
     </row>
     <row r="53" spans="1:5" ht="14.4">
-      <c r="A53" s="6"/>
+      <c r="A53" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B53" s="9" t="s">
         <v>102</v>
       </c>
@@ -2763,10 +2765,10 @@
       <c r="B56" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C56" s="33" t="s">
+      <c r="C56" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="D56" s="34"/>
+      <c r="D56" s="35"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="14.4">

</xml_diff>

<commit_message>
feat(intervals): add LC 57 Insert Interval & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E013D40-57BD-4773-A7FB-CB14D107FBB9}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61782728-07F1-4619-B2EF-3720366B8B03}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2739,7 +2739,9 @@
       <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" ht="14.4">
-      <c r="A54" s="6"/>
+      <c r="A54" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B54" s="9" t="s">
         <v>104</v>
       </c>

</xml_diff>

<commit_message>
feat(intervals): add LC 986 Interval List Intersections & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61782728-07F1-4619-B2EF-3720366B8B03}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B05AC897-8391-4058-BB5C-E15D5E75EC21}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2752,7 +2752,9 @@
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" ht="14.4">
-      <c r="A55" s="6"/>
+      <c r="A55" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B55" s="9" t="s">
         <v>106</v>
       </c>

</xml_diff>

<commit_message>
feat(linked-list): create Linked-List directory, add LC 206 Reverse Linked List & update README
</commit_message>
<xml_diff>
--- a/Copy of DSA patterns Cheat Sheet.xlsx
+++ b/Copy of DSA patterns Cheat Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3bb41df2250af5a0/Desktop/DSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B05AC897-8391-4058-BB5C-E15D5E75EC21}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="13_ncr:1_{C72A59EE-63AB-48C7-8C26-4C56EDF11D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{349F7476-C2CB-4A13-9308-1550511DFB6D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="416">
   <si>
     <t>INSTA Channel. One question Daily</t>
   </si>
@@ -2818,7 +2818,9 @@
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="14.4">
-      <c r="A61" s="6"/>
+      <c r="A61" s="6" t="s">
+        <v>415</v>
+      </c>
       <c r="B61" s="9" t="s">
         <v>117</v>
       </c>

</xml_diff>